<commit_message>
Merge complete backend implementation
Co-authored-by: Moutasem22 <44786714+Moutasem22@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/src/Hosts/SupplySonic/API/wwwroot/Uploads/addUsersSheet.xlsx
+++ b/src/Hosts/SupplySonic/API/wwwroot/Uploads/addUsersSheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25427"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FutureFace\Desktop\New folder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adham\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D81ED4FA-E028-458D-A891-F4F17D460ADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8E8957D-0C41-4BE8-8049-456045B223DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,6 +25,9 @@
     <t>Email</t>
   </si>
   <si>
+    <t>User ID</t>
+  </si>
+  <si>
     <t>Name</t>
   </si>
   <si>
@@ -44,9 +47,6 @@
   </si>
   <si>
     <t>مدير النظام</t>
-  </si>
-  <si>
-    <t>UserID</t>
   </si>
 </sst>
 </file>
@@ -121,7 +121,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:E2" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
-    <tableColumn id="8" xr3:uid="{F81143A5-C82D-454E-89CE-C057A05C3E2E}" name="UserID"/>
+    <tableColumn id="8" xr3:uid="{F81143A5-C82D-454E-89CE-C057A05C3E2E}" name="User ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Name"/>
     <tableColumn id="12" xr3:uid="{9A489230-4FEC-4BC4-A364-F30633F95686}" name="UserName"/>
     <tableColumn id="13" xr3:uid="{01DE2E8C-133E-43B8-B58E-024E25145BD0}" name="Group"/>
@@ -431,16 +431,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
         <v>3</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -451,16 +451,16 @@
         <v>11002</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>